<commit_message>
V2.0.13 FECHADA - versão a ser utilizada como código para o app - Epídio não respondeu feedback da versão V2.0.12 - whatsapp enviado em 04/08/2026
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
+++ b/V. 2 (Pudim)/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Documents\dev\Finscore\FinScore\V. 2 (Pudim)\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F78262D-6D8B-4891-929D-3AD08CD58D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B862AD-25A7-41C3-BB05-1E1B5123E2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4010788E-9D57-4518-8E30-3FC23E7ECB45}"/>
   </bookViews>
@@ -396,6 +396,1295 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Planilha1!$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>BRIGADEIRO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Planilha1!$B$4:$B$20</c:f>
+              <c:strCache>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>Callamarys</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cool Seed</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Grupo Cofesa - Super G Supermercado</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Grupo E-Construmarket - E-Construmarket Tecnologia</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Grupo E-Construmarket - Mobicloud Tecnologia</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Grupo E-Construmarket - SSA-Miro Solucoes</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Grupo Fornax - Flammers Participacoes</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Grupo Fornax - Fornax Consultoria</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Grupo Fornax - Modo Serviços RH</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Grupo Fornax - Mooven Assessoria</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Grupo JNP - JNH Hoteis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Grupo JNP - JNS Seguradora</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Grupo Mega Motos - Mega Administradora de Bens</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Grupo Mega Motos - Mega Motos Com Imp Exp</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Grupo TMDL-Log Road - Log Road Transporte Rodoviario</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Grupo TMDL-Log Road - TMDL Armazens Gerais</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>Pacto Energia</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Planilha1!$E$4:$E$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>392.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>650</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>905</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>475</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>227.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>790</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>902.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>767.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>587.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>157.5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>847.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>717.5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>295</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>855</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0429-43E4-A58E-8149C6662440}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="2087764912"/>
+        <c:axId val="2083699120"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Planilha1!$F$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>PUDIM (V2.00.07)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Planilha1!$B$4:$B$20</c:f>
+              <c:strCache>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>Callamarys</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cool Seed</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Grupo Cofesa - Super G Supermercado</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Grupo E-Construmarket - E-Construmarket Tecnologia</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Grupo E-Construmarket - Mobicloud Tecnologia</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Grupo E-Construmarket - SSA-Miro Solucoes</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Grupo Fornax - Flammers Participacoes</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Grupo Fornax - Fornax Consultoria</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Grupo Fornax - Modo Serviços RH</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Grupo Fornax - Mooven Assessoria</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Grupo JNP - JNH Hoteis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Grupo JNP - JNS Seguradora</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Grupo Mega Motos - Mega Administradora de Bens</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Grupo Mega Motos - Mega Motos Com Imp Exp</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Grupo TMDL-Log Road - Log Road Transporte Rodoviario</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Grupo TMDL-Log Road - TMDL Armazens Gerais</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>Pacto Energia</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Planilha1!$F$4:$F$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>401.22</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>644.94000000000005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>649.04</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>666.28</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>766.21</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>481.89</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>737.56</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>249.87</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>532.41</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>390.38</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>732.81</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>560.29</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>752.8</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>312.61</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0429-43E4-A58E-8149C6662440}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Planilha1!$I$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>PUDIM (V2.00.12)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Planilha1!$B$4:$B$20</c:f>
+              <c:strCache>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>Callamarys</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Cool Seed</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Grupo Cofesa - Super G Supermercado</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Grupo E-Construmarket - E-Construmarket Tecnologia</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Grupo E-Construmarket - Mobicloud Tecnologia</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Grupo E-Construmarket - SSA-Miro Solucoes</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Grupo Fornax - Flammers Participacoes</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Grupo Fornax - Fornax Consultoria</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Grupo Fornax - Modo Serviços RH</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Grupo Fornax - Mooven Assessoria</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Grupo JNP - JNH Hoteis</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Grupo JNP - JNS Seguradora</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Grupo Mega Motos - Mega Administradora de Bens</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Grupo Mega Motos - Mega Motos Com Imp Exp</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Grupo TMDL-Log Road - Log Road Transporte Rodoviario</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Grupo TMDL-Log Road - TMDL Armazens Gerais</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>Pacto Energia</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Planilha1!$I$4:$I$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>394.43</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>731.87</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>726.56</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>747.93</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>897.64</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>854.01</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>244.87</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>602.53</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>376.14</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>845.81</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>621.24</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>837.55</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>289.87</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-0429-43E4-A58E-8149C6662440}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="2087764912"/>
+        <c:axId val="2083699120"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2087764912"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2083699120"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2083699120"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2087764912"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>531948</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>161470</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>281213</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>81642</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46ECCCF6-9CAD-1E7A-4F7C-42D6658CC089}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -781,7 +2070,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="5" t="str">
-        <f>_xlfn.CONCAT(A4,RIGHT(B4,30))</f>
+        <f t="shared" ref="C4:C20" si="0">_xlfn.CONCAT(A4,RIGHT(B4,30))</f>
         <v>1Callamarys</v>
       </c>
       <c r="D4" s="14" t="s">
@@ -817,7 +2106,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="str">
-        <f>_xlfn.CONCAT(A5,RIGHT(B5,30))</f>
+        <f t="shared" si="0"/>
         <v>2Cool Seed</v>
       </c>
       <c r="D5" s="14" t="s">
@@ -853,7 +2142,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="5" t="str">
-        <f>_xlfn.CONCAT(A6,RIGHT(B6,30))</f>
+        <f t="shared" si="0"/>
         <v>3 Cofesa - Super G Supermercado</v>
       </c>
       <c r="D6" s="14" t="s">
@@ -889,7 +2178,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="5" t="str">
-        <f>_xlfn.CONCAT(A7,RIGHT(B7,30))</f>
+        <f t="shared" si="0"/>
         <v>4t - E-Construmarket Tecnologia</v>
       </c>
       <c r="D7" s="14" t="s">
@@ -925,7 +2214,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="5" t="str">
-        <f>_xlfn.CONCAT(A8,RIGHT(B8,30))</f>
+        <f t="shared" si="0"/>
         <v>5umarket - Mobicloud Tecnologia</v>
       </c>
       <c r="D8" s="14" t="s">
@@ -961,7 +2250,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="5" t="str">
-        <f>_xlfn.CONCAT(A9,RIGHT(B9,30))</f>
+        <f t="shared" si="0"/>
         <v>6strumarket - SSA-Miro Solucoes</v>
       </c>
       <c r="D9" s="14" t="s">
@@ -997,7 +2286,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="5" t="str">
-        <f>_xlfn.CONCAT(A10,RIGHT(B10,30))</f>
+        <f t="shared" si="0"/>
         <v>7ornax - Flammers Participacoes</v>
       </c>
       <c r="D10" s="14" t="s">
@@ -1036,7 +2325,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="5" t="str">
-        <f>_xlfn.CONCAT(A11,RIGHT(B11,30))</f>
+        <f t="shared" si="0"/>
         <v>8po Fornax - Fornax Consultoria</v>
       </c>
       <c r="D11" s="14" t="s">
@@ -1072,7 +2361,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="5" t="str">
-        <f>_xlfn.CONCAT(A12,RIGHT(B12,30))</f>
+        <f t="shared" si="0"/>
         <v>9rupo Fornax - Modo Serviços RH</v>
       </c>
       <c r="D12" s="14" t="s">
@@ -1108,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="5" t="str">
-        <f>_xlfn.CONCAT(A13,RIGHT(B13,30))</f>
+        <f t="shared" si="0"/>
         <v>10upo Fornax - Mooven Assessoria</v>
       </c>
       <c r="D13" s="14" t="s">
@@ -1144,7 +2433,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="5" t="str">
-        <f>_xlfn.CONCAT(A14,RIGHT(B14,30))</f>
+        <f t="shared" si="0"/>
         <v>11Grupo JNP - JNH Hoteis</v>
       </c>
       <c r="D14" s="14" t="s">
@@ -1180,7 +2469,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="5" t="str">
-        <f>_xlfn.CONCAT(A15,RIGHT(B15,30))</f>
+        <f t="shared" si="0"/>
         <v>12Grupo JNP - JNS Seguradora</v>
       </c>
       <c r="D15" s="14" t="s">
@@ -1216,7 +2505,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="5" t="str">
-        <f>_xlfn.CONCAT(A16,RIGHT(B16,30))</f>
+        <f t="shared" si="0"/>
         <v>13 - Mega Administradora de Bens</v>
       </c>
       <c r="D16" s="14" t="s">
@@ -1252,7 +2541,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="5" t="str">
-        <f>_xlfn.CONCAT(A17,RIGHT(B17,30))</f>
+        <f t="shared" si="0"/>
         <v>14Motos - Mega Motos Com Imp Exp</v>
       </c>
       <c r="D17" s="14" t="s">
@@ -1288,7 +2577,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="5" t="str">
-        <f>_xlfn.CONCAT(A18,RIGHT(B18,30))</f>
+        <f t="shared" si="0"/>
         <v>15Log Road Transporte Rodoviario</v>
       </c>
       <c r="D18" s="14" t="s">
@@ -1327,7 +2616,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="5" t="str">
-        <f>_xlfn.CONCAT(A19,RIGHT(B19,30))</f>
+        <f t="shared" si="0"/>
         <v>16og Road - TMDL Armazens Gerais</v>
       </c>
       <c r="D19" s="14" t="s">
@@ -1363,7 +2652,7 @@
         <v>3</v>
       </c>
       <c r="C20" s="5" t="str">
-        <f>_xlfn.CONCAT(A20,RIGHT(B20,30))</f>
+        <f t="shared" si="0"/>
         <v>17Pacto Energia</v>
       </c>
       <c r="D20" s="14" t="s">
@@ -1394,5 +2683,6 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>